<commit_message>
citations.xlsx: 추가일 정렬 반영 (556건)
</commit_message>
<xml_diff>
--- a/nm-reference/citations.xlsx
+++ b/nm-reference/citations.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -46,8 +48,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -31106,6 +31109,9 @@
           <t>10.21097/ksw.2026.5.21.2.105</t>
         </is>
       </c>
+      <c r="G542" s="1" t="n">
+        <v>46204</v>
+      </c>
       <c r="H542" t="inlineStr">
         <is>
           <t>본 연구의 목적은 키워드 네트워크 분석과 토픽모델링을 활용하여 청년 1인가구를 주제로 한 국내 학술 연구의 동향을 체계적으로 분석하는 것이다. 이를 위해 NetMiner 4.5.1의 확장 프로그램인 Biblio Data Collector(이하 BDC)를 통해 수집한 논문 95편을 대상으로 키워드 빈도분석, 동시출현 빈도분석, 중심성 분석, 토픽모델링을 수행하였다. 연구의 결과 첫째, 빈도분석에서는 우울, 주거환경, 소득, 공유주택, 외로움 순으로 높은 빈도를 보였다. 둘째, 동시출현 빈도분석에서는 라이프스타일-삶의 만족도이 가장 높은 동시출현 빈도를 보였다. 셋째, 중심성 분석에서는 우울과 주거환경이 연결·근접·매개중심성 모두에서 1, 2위를 차지하여 연구 네트워크의 핵심 허브 역할을 담당하고 있음이 확인되었다. 넷째, 토픽모델링 분석에서는 정신건강과 심리적 특성, 일상생활과 사회적 지지, 사회적 고립과 심리적 위기, 외로움과 사회적 자원 부족, 코로나19 전후 생활 변화와 건강, 대안적 주거 환경과 주거 만족의 6개 토픽이 도출되었다. 본 연구의 결과는 청년 1인가구 후속 연구를 위한 기초자료를 제공하고, 청년 1인가구를 위한 정책 마련에 기여할 것으로 보인다.</t>
@@ -31155,6 +31161,9 @@
       <c r="E543" t="n">
         <v>2026</v>
       </c>
+      <c r="G543" s="1" t="n">
+        <v>46204</v>
+      </c>
       <c r="H543" t="inlineStr">
         <is>
           <t>본 연구는 최근 10년간 국내 아동 구강건강 관련 연구를 대상으로 텍스트 네트워크 분석을 수행하여 주요 연구 주제와 지식 구조를 규명하고자 하였다. 연구대상은 학술연구정보서비스에서 아동과 구강을 검색어로 하여 최근 10년, KCI 등재, 한국어, 원문 제공 조건을 충족하는 44편의 논문이다. 수집된 논문의 키워드를 정제한 후 NetMiner 4 프로그램을 활용하여 키워드 빈도분석, 연결중심성 분석, 네트워크 군집분석을 수행하였다. 연구결과, 키워드 빈도분석에서는 아동, 구강건강이 가장 높은 빈도로 나타났고, 구강건강조사, 치아우식증, 칫솔질, 구강운동기능 등이 주요 키워드로 확인되었다. 연결중심성 분석에서는 아동, 구강건강, 치아우식증, 구강건강행동, 부모가 핵심 노드로 나타나 아동 구강건강 연구가 질병, 행동, 보호자 요인을 중심으로 전개되고 있음을 확인하였다. 군집분석 결과, 연구 주제는 치아우식증 및 구강질환, 구강건강행동 및 부모 요인, 장애 아동 구강기능·중재, 구강보건교육 예방·관리의 네 가지 영역으로 구조화되었다. 한편 디지털 헬스케어 및 인공지능 관련 키워드는 주요 네트워크에서 명확하게 확인되지 않아 해당 분야 연구가 제한적인 것으로 확인되었다. 본 연구는 국내 아동 구강건강 연구의 지식구조를 체계적으로 제시하고, 분석 결과를 기반으로 인공지능 기반 구강관리 전략의 적용 방향을 제언하였다는 점에 의의가 있다.</t>
@@ -31208,6 +31217,9 @@
         <is>
           <t>10.14333/kjte.2026.42.3.31</t>
         </is>
+      </c>
+      <c r="G544" s="1" t="n">
+        <v>46204</v>
       </c>
       <c r="H544" t="inlineStr">
         <is>
@@ -31299,6 +31311,9 @@
           <t>10.5334/ijic.9045</t>
         </is>
       </c>
+      <c r="G546" s="1" t="n">
+        <v>46198</v>
+      </c>
       <c r="H546" t="inlineStr">
         <is>
           <t>Objectives: Despite the significant advantages of public-private partnerships (PPPs), understanding of the organisational roles that shape partnership functioning within integrated care networks remains limited. This study investigated the structural characteristics of PPPs and identified organisational roles within an integrated care network in a Seoul district, Korea.Methods: Using the 2020 Integrated Care Network Survey, this study analyzed modularity, eigenvector centrality, and brokerage in 82 public and private organisations across five different types: district offices, public health centres, healthcare institutions, social welfare institutions, and community organisations. Results: Our results reveal that integrated care organisations are predominantly divided into two major networks: disability care and elderly care. The highest centrality in the elderly care network is occupied by the dementia relief centre and social welfare institutions, while the disability care network is dominated by public institutions, the Health and Welfare Cooperative, and a social service centre for the disabled. Regarding organisational roles, social welfare institutions function primarily as coordinators, representatives, and gatekeepers, whereas public institutions-including district offices, public health centres, and community service centres-serve as consultants and liaisons. Notably, public institutions assume more prominent roles and private organisations demonstrate less involvement in the disability care network compared to the elderly care network. Conclusion: These findings underscore the importance of defining clear organisational roles and interaction mechanisms between public and private sectors, offering valuable insights for policy design aimed at enhancing coordination, accountability, and sustainability within PPP-based integrated care systems.</t>
@@ -31347,6 +31362,9 @@
       </c>
       <c r="E547" t="n">
         <v>2026</v>
+      </c>
+      <c r="G547" s="1" t="n">
+        <v>46204</v>
       </c>
       <c r="H547" t="inlineStr">
         <is>
@@ -31405,6 +31423,9 @@
           <t>10.22718/kga.2026.10.2.019</t>
         </is>
       </c>
+      <c r="G548" s="1" t="n">
+        <v>46204</v>
+      </c>
       <c r="H548" t="inlineStr">
         <is>
           <t>본 연구는 키워드 네트워크 분석과 토픽모델링을 활용하여 국내 노인 1인가구 관련 연구동향을 분석하는 데 목적이 있다. 이를 위해 국내 KCI 등재(후보) 학술지에 게재된 노인 1인가구 관련 논문 111편을 대상으로 넷마이너(NetMiner 4)를 이용하여 키워드 네트워크 분석과 토픽모델링을 수행하였다. 키워드 네트워크 분석에서는 키워드 빈도분석과 동시출현 분석을 실시하고 연결중심성, 근접중심성, 매개중심성을 산출하여 핵심 개념의 구조를 분석하였다. 분석 결과, 사회적 관계, 우울, 정책, 지원, 삶의 만족 등이 주요 키워드로 나타났다. 토픽모델링 분석에서는 총 4개의 토픽이 도출되었다. 토픽-1은 사회적 지지와 돌봄을 통한 노년기 삶의 질, 토픽-2는 경제 및 주거 조건과 빈곤 문제, 토픽-3은 사회참여와 공동체 활동을 통한 능동적 삶, 토픽-4는 우울과 건강 상태를 중심으로 한 심리·정서적 위기와 관련된 주제로 나타났다. 이러한 결과는 노인 1인가구 연구가 경제적 조건과 사회적 관계를 중심으로 사회참여와 정신건강 등 다양한 주제로 확장되어 왔음을 보여준다. 본 연구는 국내 노인 1인가구 연구의 주요 주제와 지식 구조를 체계적으로 제시하고, 향후 연구 방향을 위한 기초자료를 제공한다는 점에서 의의를 가진다.</t>
@@ -31459,6 +31480,9 @@
           <t>10.22173/ksss.2026.39.specialissue.6</t>
         </is>
       </c>
+      <c r="G549" s="1" t="n">
+        <v>46204</v>
+      </c>
       <c r="H549" t="inlineStr">
         <is>
           <t>본 연구는 학교스포츠클럽 관련 언론 보도의 변화를 텍스트 마이닝 기법을 활용하여 분석하였다. 2007년부터 2023년까지 빅카인즈를 통해 수집된 7,922개의 언론 보도 기사를 바탕으로 27,286개의 키워드를 추출하고, 시기별(1기: 2007- 2011, 2기: 2012-2018, 3기: 2019-2023) 핵심 주제어의 변화를 분석하였다. 넷마이너 4.5 프로그램을 사용하여 TF-IDF 분석, 의미연결망 분석 및 네트워크 시각화 분석을 수행하였다. 이를 통해 도출된 결론은 다음과 같다. TF-IDF 분석에서는 제1기에는 체육, 참여, 지원 등이, 제2기에는 교육, 지역, 종목 등이, 제3기에는 건강, 체력, 코로나 등이 중요한 키워드로 도출되어 시기별 관심 주제의 차이를 확인할 수 있었다. 의미연결망 분석에서는 제1기에는 스포츠, 체육, 학교, 학생, 교육, 운영, 활성, 건강, 참여 순으로 높은 연결 중심성 지수가 나타났다. 제2기에는 스포츠, 학교, 학생, 활동, 대회, 인성, 폭력, 여학생, 시설 등의 순으로 중심성이 높게 나타났다. 제3기에는 스포츠, 체육, 학교, 학생, 건강, 대회, 코로나, 운동, 온라인, 소통 등의 순으로 연결 중심성이 확인되었다. 이를 통해 학교스포츠클럽 관련 언론 보도는 시기별 정책 환경과 사회적 이슈 변화에 따라 핵심 키워드와 연결 구조가 달라졌음을 확인하였다.</t>
@@ -31545,6 +31569,9 @@
         <is>
           <t>10.1136/bmjopen-2025-101505</t>
         </is>
+      </c>
+      <c r="G551" s="1" t="n">
+        <v>46198</v>
       </c>
       <c r="H551" t="inlineStr">
         <is>
@@ -31783,6 +31810,9 @@
       <c r="E555" t="n">
         <v>2026</v>
       </c>
+      <c r="G555" s="1" t="n">
+        <v>46204</v>
+      </c>
       <c r="H555" t="inlineStr">
         <is>
           <t>Purpose : This study aimed to examine research trends and explore the conceptual structure of employment preparation stress among nursing students using text network analysis and topic modeling. Methods : A descriptive study was conducted based on the abstracts of 39 Korean studies published between 2015 and 2024.
@@ -31837,6 +31867,9 @@
         <is>
           <t>10.24881/tjk.2026.17.2.131</t>
         </is>
+      </c>
+      <c r="G556" s="1" t="n">
+        <v>46204</v>
       </c>
       <c r="H556" t="inlineStr">
         <is>
@@ -31895,6 +31928,9 @@
           <t>10.35734/karp.2026.33.2.007</t>
         </is>
       </c>
+      <c r="G557" s="1" t="n">
+        <v>46204</v>
+      </c>
       <c r="H557" t="inlineStr">
         <is>
           <t>본 연구는 키워드 네트워크 분석과 토픽모델링을 활용하여 국내 학술지에 게재된 집단상담 관련 연구동향을 분석하는 데 목적이 있다. 이를 위하여 국내 등재 학술지에 게재된 910편의 논문을 분석하였다. 논문 분석을 위하여 넷마이너(NetMiner) 4.5 프로그램을 활용하여 논문에 잠재된 토픽과 키워드를 도출하였다. 본 연구는 전기(2000년-2010년)와 후기(2011-2022년)로 나누어 토픽모델링을 분석하고 토픽 분류결과 동일하게 나타난 토픽 간 연결중심성과 상위단어들의 동시출현단어들을 분석하였다. 또한 전체 집단상담에 대한 토픽 변화추이를 분석하여 연구 주제가 시간 추이에 따라 어떻게 변화하는지를 살펴보았다. 분석결과, 전기에는 학교생활적응 개입, 정서조절 및 적응 개입, 부적응과 가족 요인 개입, 인터넷중독 개입, 진로 개입, 정신건강 개입 등의 토픽이 도출되었으며, 후기에는 정신건강 개입, 정서조절 및 적응 개입, 진로 개입, 매체중독 개입 등의 토픽이 주요 연구주제로 나타났다. 또한 시기별 토픽 추이 분석 결과, 진로 개입과 정서조절 및 적응 개입은 전 기간에 걸쳐 지속적으로 나타난 주요 연구주제로 확인되었으며, 최근에는 정신건강 및 매체중독 관련 연구의 증가가 확인되었다. 이상의 분석결과와 논의를 바탕으로 향후 집단상담 연구에 대한 시사점을 제시하였다.</t>

</xml_diff>

<commit_message>
Auto: NetMiner citations update 2026-07 (monthly)
</commit_message>
<xml_diff>
--- a/nm-reference/citations.xlsx
+++ b/nm-reference/citations.xlsx
@@ -522,6 +522,11 @@
       <c r="E2" t="n">
         <v>2026</v>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>10.52902/kjsc.2026.56.35</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>본 연구는 간호대학생의 환자안전역량 관련 연구의 동향과 지식구조를 체계적으로 규명하기 위하여 텍스트 네트워크 분석과 토픽모델링을 적용한 이차자료 분석 연구이다. 기존 연구들이 개별 변수 간 관계나 교육 중재 효과를 중심으로 수행된 것과 달리, 본 연구는 연구 분야 전반의 구조적 특성과 핵심 주제를 통합적으로 파악하고자 하였다. 2015년부터 2025년까지 국내 주요 학술 데이터베이스(RISS, KISS, DBpia, NDSL, KCI)를 통해 검색된 24편의 논문을 대상으로 포함 및 제외 기준을 적용하여 분석하였다. 선정된 논문의 제목, 초록 및 저자 키워드를 수집하여 전처리한 후 NetMiner 4.0을 활용한 키워드 동시출현 네트워크 분석과 잠재 디리클레 할당(LDA) 기반 토픽모델링을 수행하였다. 분석 결과, ‘환자안전역량’을 중심으로 ‘비판적사고’, ‘환자안전관리’, ‘시뮬레이션’, ‘안전간호수행’, ‘환자안전교육’, ‘안전행동’, ‘의사소통’이 핵심적으로 연결된 네트워크 구조가 확인되었다. 또한 토픽모델링을 통해 환자안전교육, 임상추론 및 문제해결, 의사소통 및 팀워크, 환자안전 인식 및 태도, 환자안전행동의 5개 주요 연구 주제가 도출되었다. 이는 간호대학생의 환자안전역량 연구가 인지적 역량과 교육적 경험을 중심으로 구조화되어 있으며, 협력적 실무 역량이 이를 통합하는 핵심 요소임을 시사한다. 본 연구는 환자안전역량 연구의 지식구조를 구조적으로 제시함으로써 향후 연구 방향 설정과 교육전략 수립에 중요한 근거를 제공한다. 또한 비판적사고, 시뮬레이션 기반 학습, 의사소통 및 팀워크를 통합한 교육전략과 함께 교육과 임상 환경을 연계하는 정책적 지원의 필요성을 제시한다.</t>
@@ -543,7 +548,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>검증필요</t>
+          <t>활용</t>
         </is>
       </c>
     </row>
@@ -570,6 +575,11 @@
       </c>
       <c r="E3" t="n">
         <v>2026</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>10.16980/jitc.22.3.202606.519</t>
+        </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -598,7 +608,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>검증필요</t>
+          <t>활용</t>
         </is>
       </c>
     </row>
@@ -626,6 +636,11 @@
       <c r="E4" t="n">
         <v>2026</v>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>10.16881/jss.2026.07.37.3.311</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>본 연구는 키워드 네트워크 분석을 통하여 국내 트라우마 연구의 동향을 살펴보는 데 목적을 두었다. 이를 위해 국내 학술지에 게재된 트라우마 관련 연구논문을 수집하고, 논문에 제시된 키워드를 추출하였다. 자료 수집 및 분석을 위해 NetMiner 4.5 프로그램을 활용하여 키워드 간 공출현 빈도와 네트워크 구조를 분석하였다. 연구결과는 다음과 같다. 첫째, 트라우마 연구에서 빈도 상위 키워드는 외상 후 성장, 질적연구, 외상 후 스트레스장애, 청소년, 트라우마 경험, 치유 등의 순으로 나타났다. 둘째, 연결중심성과 매개중심성이 높은 키워드는 외상 후 성장과 외상 후 스트레스 장애로 나타나 트라우마 연구에서 핵심적인 역할을 하는 개념임을 확인할 수 있었다. 셋째, 외상 후 성장과 외상 후 스트레스 장애를 중심으로 한 에고 네트워크 분석 결과 다양한 치료 접근과 대상 집단이 연결되어 나타나 트라우마 연구가 회복과 개입, 사회적 맥락을 함께 다루고 있음을 확인할 수 있었다. 넷째, Cluster 분석 결과 외상 경험과 증상, 치유와 개입, 사회적 사건과 대상 집단의 세 가지 주제 영역을 중심으로 연구가 이루어지고 있는 것으로 나타났다. 이러한 연구 결과를 바탕으로 트라우마 연구의 주요 지식구조를 파악하고 향후 연구 방향과 상담학적 시사점을 제시하였다.</t>
@@ -647,7 +662,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>검증필요</t>
+          <t>활용</t>
         </is>
       </c>
     </row>
@@ -863,7 +878,7 @@
         <v>1</v>
       </c>
       <c r="N8" t="n">
-        <v>11.7155</v>
+        <v>9.1409</v>
       </c>
       <c r="O8" t="n">
         <v>1</v>
@@ -1310,7 +1325,7 @@
         <v>4</v>
       </c>
       <c r="N16" t="n">
-        <v>53.1893</v>
+        <v>46.8229</v>
       </c>
       <c r="O16" t="n">
         <v>4</v>
@@ -1364,7 +1379,7 @@
         <v>2</v>
       </c>
       <c r="N17" t="n">
-        <v>18.7673</v>
+        <v>14.5326</v>
       </c>
       <c r="O17" t="n">
         <v>2</v>
@@ -1961,13 +1976,13 @@
         </is>
       </c>
       <c r="K28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N28" t="n">
-        <v>0</v>
+        <v>7.2188</v>
       </c>
       <c r="O28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P28" t="inlineStr">
         <is>
@@ -3383,7 +3398,7 @@
         <v>2</v>
       </c>
       <c r="N53" t="n">
-        <v>4.1242</v>
+        <v>2.9536</v>
       </c>
       <c r="O53" t="n">
         <v>2</v>
@@ -3482,13 +3497,13 @@
         </is>
       </c>
       <c r="K55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N55" t="n">
-        <v>0.9712</v>
+        <v>1.6991</v>
       </c>
       <c r="O55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P55" t="inlineStr">
         <is>
@@ -4222,7 +4237,7 @@
         <v>1</v>
       </c>
       <c r="N68" t="n">
-        <v>0.6688</v>
+        <v>0.5872000000000001</v>
       </c>
       <c r="O68" t="n">
         <v>1</v>
@@ -7911,7 +7926,7 @@
         <v>16</v>
       </c>
       <c r="N131" t="n">
-        <v>7.0897</v>
+        <v>6.368</v>
       </c>
       <c r="O131" t="n">
         <v>16</v>
@@ -7962,7 +7977,7 @@
         <v>4</v>
       </c>
       <c r="N132" t="n">
-        <v>1.9752</v>
+        <v>1.9216</v>
       </c>
       <c r="O132" t="n">
         <v>4</v>
@@ -8072,7 +8087,7 @@
         <v>4</v>
       </c>
       <c r="N134" t="n">
-        <v>1.1151</v>
+        <v>0.9709</v>
       </c>
       <c r="O134" t="n">
         <v>4</v>
@@ -8196,7 +8211,7 @@
         <v>0</v>
       </c>
       <c r="N136" t="n">
-        <v>0.6614</v>
+        <v>0.6504</v>
       </c>
       <c r="O136" t="n">
         <v>8</v>
@@ -8263,7 +8278,7 @@
         <v>0</v>
       </c>
       <c r="N137" t="n">
-        <v>0.8303</v>
+        <v>0.796</v>
       </c>
       <c r="O137" t="n">
         <v>4</v>
@@ -8829,7 +8844,7 @@
         <v>1</v>
       </c>
       <c r="N147" t="n">
-        <v>0.8238</v>
+        <v>0.7734</v>
       </c>
       <c r="O147" t="n">
         <v>1</v>
@@ -8960,7 +8975,7 @@
         <v>0</v>
       </c>
       <c r="N149" t="n">
-        <v>0.4431</v>
+        <v>0.4056</v>
       </c>
       <c r="O149" t="n">
         <v>2</v>
@@ -9027,7 +9042,7 @@
         <v>0</v>
       </c>
       <c r="N150" t="n">
-        <v>0.4431</v>
+        <v>0.4245</v>
       </c>
       <c r="O150" t="n">
         <v>3</v>
@@ -9078,7 +9093,7 @@
         <v>1</v>
       </c>
       <c r="N151" t="n">
-        <v>0.2044</v>
+        <v>0.1527</v>
       </c>
       <c r="O151" t="n">
         <v>1</v>
@@ -12035,13 +12050,13 @@
         </is>
       </c>
       <c r="K204" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N204" t="n">
-        <v>0</v>
+        <v>0.4056</v>
       </c>
       <c r="O204" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P204" t="inlineStr">
         <is>
@@ -12861,7 +12876,7 @@
         <v>0</v>
       </c>
       <c r="N218" t="n">
-        <v>0.7758</v>
+        <v>0.742</v>
       </c>
       <c r="O218" t="n">
         <v>5</v>
@@ -12909,13 +12924,13 @@
         </is>
       </c>
       <c r="K219" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N219" t="n">
-        <v>2.1617</v>
+        <v>3.2467</v>
       </c>
       <c r="O219" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P219" t="inlineStr">
         <is>
@@ -13195,7 +13210,7 @@
         <v>4</v>
       </c>
       <c r="N224" t="n">
-        <v>0.9579</v>
+        <v>0.9455</v>
       </c>
       <c r="O224" t="n">
         <v>4</v>
@@ -13243,13 +13258,13 @@
         </is>
       </c>
       <c r="K225" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N225" t="n">
-        <v>0.7207</v>
+        <v>0.9466</v>
       </c>
       <c r="O225" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P225" t="inlineStr">
         <is>
@@ -13297,7 +13312,7 @@
         <v>1</v>
       </c>
       <c r="N226" t="n">
-        <v>1.9609</v>
+        <v>1.9705</v>
       </c>
       <c r="O226" t="n">
         <v>1</v>
@@ -13658,7 +13673,7 @@
         <v>2</v>
       </c>
       <c r="N232" t="n">
-        <v>0.8791</v>
+        <v>0.8588</v>
       </c>
       <c r="O232" t="n">
         <v>2</v>
@@ -13709,7 +13724,7 @@
         <v>2</v>
       </c>
       <c r="N233" t="n">
-        <v>0.4789</v>
+        <v>0.4728</v>
       </c>
       <c r="O233" t="n">
         <v>2</v>
@@ -13757,13 +13772,13 @@
         </is>
       </c>
       <c r="K234" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N234" t="n">
-        <v>0.4789</v>
+        <v>0.7114</v>
       </c>
       <c r="O234" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P234" t="inlineStr">
         <is>
@@ -14856,7 +14871,7 @@
         <v>1</v>
       </c>
       <c r="N253" t="n">
-        <v>0.3288</v>
+        <v>0.3239</v>
       </c>
       <c r="O253" t="n">
         <v>1</v>
@@ -17104,7 +17119,7 @@
         <v>2</v>
       </c>
       <c r="N292" t="n">
-        <v>0.6283</v>
+        <v>0.6257</v>
       </c>
       <c r="O292" t="n">
         <v>2</v>
@@ -17219,13 +17234,13 @@
         </is>
       </c>
       <c r="K294" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="N294" t="n">
-        <v>1.4371</v>
+        <v>1.4293</v>
       </c>
       <c r="O294" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="P294" t="inlineStr">
         <is>
@@ -17289,7 +17304,7 @@
         <v>0</v>
       </c>
       <c r="N295" t="n">
-        <v>3.5686</v>
+        <v>3.4879</v>
       </c>
       <c r="O295" t="n">
         <v>45</v>
@@ -17337,13 +17352,13 @@
         </is>
       </c>
       <c r="K296" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N296" t="n">
-        <v>5.1194</v>
+        <v>4.9612</v>
       </c>
       <c r="O296" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="P296" t="inlineStr">
         <is>
@@ -17501,7 +17516,7 @@
         <v>15</v>
       </c>
       <c r="N299" t="n">
-        <v>5.282</v>
+        <v>5.2024</v>
       </c>
       <c r="O299" t="n">
         <v>15</v>
@@ -17770,7 +17785,7 @@
         <v>8</v>
       </c>
       <c r="N304" t="n">
-        <v>2.1818</v>
+        <v>2.2603</v>
       </c>
       <c r="O304" t="n">
         <v>8</v>
@@ -17837,7 +17852,7 @@
         <v>0</v>
       </c>
       <c r="N305" t="n">
-        <v>0.9684</v>
+        <v>0.9699</v>
       </c>
       <c r="O305" t="n">
         <v>9</v>
@@ -17895,7 +17910,7 @@
         </is>
       </c>
       <c r="K306" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L306" t="n">
         <v>7</v>
@@ -17907,7 +17922,7 @@
         <v>1.9765</v>
       </c>
       <c r="O306" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="P306" t="inlineStr">
         <is>
@@ -18615,13 +18630,13 @@
         </is>
       </c>
       <c r="K318" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N318" t="n">
-        <v>0.9686</v>
+        <v>0.9752999999999999</v>
       </c>
       <c r="O318" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P318" t="inlineStr">
         <is>
@@ -19012,7 +19027,7 @@
         <v>4</v>
       </c>
       <c r="N325" t="n">
-        <v>0.7744</v>
+        <v>0.7703</v>
       </c>
       <c r="O325" t="n">
         <v>4</v>
@@ -19063,7 +19078,7 @@
         <v>5</v>
       </c>
       <c r="N326" t="n">
-        <v>0.451</v>
+        <v>0.45</v>
       </c>
       <c r="O326" t="n">
         <v>5</v>
@@ -19786,7 +19801,7 @@
         <v>2</v>
       </c>
       <c r="N339" t="n">
-        <v>0.2831</v>
+        <v>0.2835</v>
       </c>
       <c r="O339" t="n">
         <v>2</v>
@@ -19904,7 +19919,7 @@
         <v>2</v>
       </c>
       <c r="N341" t="n">
-        <v>0.0813</v>
+        <v>0.0808</v>
       </c>
       <c r="O341" t="n">
         <v>2</v>
@@ -21507,13 +21522,13 @@
         </is>
       </c>
       <c r="K372" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="N372" t="n">
-        <v>13.0126</v>
+        <v>17.688</v>
       </c>
       <c r="O372" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P372" t="inlineStr">
         <is>
@@ -21561,7 +21576,7 @@
         <v>19</v>
       </c>
       <c r="N373" t="n">
-        <v>4.2495</v>
+        <v>4.3259</v>
       </c>
       <c r="O373" t="n">
         <v>19</v>
@@ -22324,7 +22339,7 @@
         <v>7</v>
       </c>
       <c r="N386" t="n">
-        <v>2.0742</v>
+        <v>2.1594</v>
       </c>
       <c r="O386" t="n">
         <v>7</v>
@@ -22442,7 +22457,7 @@
         <v>9</v>
       </c>
       <c r="N388" t="n">
-        <v>0.3798</v>
+        <v>0.3805</v>
       </c>
       <c r="O388" t="n">
         <v>9</v>
@@ -24071,13 +24086,13 @@
         </is>
       </c>
       <c r="K416" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N416" t="n">
-        <v>0.3878</v>
+        <v>0.3789</v>
       </c>
       <c r="O416" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P416" t="inlineStr">
         <is>
@@ -24125,7 +24140,7 @@
         <v>2</v>
       </c>
       <c r="N417" t="n">
-        <v>0.3798</v>
+        <v>0.3789</v>
       </c>
       <c r="O417" t="n">
         <v>2</v>
@@ -25953,7 +25968,7 @@
         <v>17</v>
       </c>
       <c r="N451" t="n">
-        <v>4.3538</v>
+        <v>4.4885</v>
       </c>
       <c r="O451" t="n">
         <v>17</v>
@@ -27541,13 +27556,13 @@
         </is>
       </c>
       <c r="K477" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N477" t="n">
-        <v>0.3538</v>
+        <v>0.3443</v>
       </c>
       <c r="O477" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="P477" t="inlineStr">
         <is>
@@ -27595,7 +27610,7 @@
         <v>5</v>
       </c>
       <c r="N478" t="n">
-        <v>1.1189</v>
+        <v>1.1408</v>
       </c>
       <c r="O478" t="n">
         <v>5</v>
@@ -29920,7 +29935,7 @@
         <v>66</v>
       </c>
       <c r="N519" t="n">
-        <v>1.8142</v>
+        <v>1.7677</v>
       </c>
       <c r="O519" t="n">
         <v>66</v>
@@ -30003,13 +30018,13 @@
         </is>
       </c>
       <c r="K520" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N520" t="n">
-        <v>6.2918</v>
+        <v>6.3235</v>
       </c>
       <c r="O520" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="P520" t="inlineStr">
         <is>
@@ -30057,7 +30072,7 @@
         <v>17</v>
       </c>
       <c r="N521" t="n">
-        <v>1.723</v>
+        <v>1.6771</v>
       </c>
       <c r="O521" t="n">
         <v>17</v>
@@ -30133,7 +30148,7 @@
         <v>10</v>
       </c>
       <c r="N522" t="n">
-        <v>6.2116</v>
+        <v>6.0624</v>
       </c>
       <c r="O522" t="n">
         <v>10</v>
@@ -30269,7 +30284,7 @@
         <v>3</v>
       </c>
       <c r="N524" t="n">
-        <v>0.217</v>
+        <v>0.2169</v>
       </c>
       <c r="O524" t="n">
         <v>3</v>
@@ -30432,7 +30447,7 @@
         <v>1</v>
       </c>
       <c r="N527" t="n">
-        <v>0.3944</v>
+        <v>0.3962</v>
       </c>
       <c r="O527" t="n">
         <v>1</v>
@@ -30975,7 +30990,7 @@
         <v>331</v>
       </c>
       <c r="N539" t="n">
-        <v>36.6041</v>
+        <v>37.0458</v>
       </c>
       <c r="O539" t="n">
         <v>331</v>
@@ -31123,7 +31138,7 @@
         <v>33</v>
       </c>
       <c r="N542" t="n">
-        <v>3.1998</v>
+        <v>3.1147</v>
       </c>
       <c r="O542" t="n">
         <v>33</v>
@@ -31179,7 +31194,7 @@
         <v>4</v>
       </c>
       <c r="N543" t="n">
-        <v>0.6822</v>
+        <v>0.6844</v>
       </c>
       <c r="O543" t="n">
         <v>4</v>
@@ -31585,7 +31600,7 @@
         <v>80</v>
       </c>
       <c r="N553" t="n">
-        <v>14.4577</v>
+        <v>13.7236</v>
       </c>
       <c r="O553" t="n">
         <v>80</v>
@@ -31641,7 +31656,7 @@
         <v>22</v>
       </c>
       <c r="N554" t="n">
-        <v>0.949</v>
+        <v>0.9577</v>
       </c>
       <c r="O554" t="n">
         <v>22</v>
@@ -31697,7 +31712,7 @@
         <v>9</v>
       </c>
       <c r="N555" t="n">
-        <v>0.7161</v>
+        <v>0.7188</v>
       </c>
       <c r="O555" t="n">
         <v>9</v>
@@ -31753,7 +31768,7 @@
         <v>5</v>
       </c>
       <c r="N556" t="n">
-        <v>2.2427</v>
+        <v>2.246</v>
       </c>
       <c r="O556" t="n">
         <v>5</v>

</xml_diff>